<commit_message>
feat: añadir informe final en PDF
</commit_message>
<xml_diff>
--- a/excel/cartera_sp500.xlsx
+++ b/excel/cartera_sp500.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acus Nervus\Desktop\sp500-cartera-analisis\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{137554EE-C9EF-435A-996E-EBCA6AF47300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C838E2B-5F68-4CDD-972D-2F1C0840DE7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14385" yWindow="45" windowWidth="14415" windowHeight="15390" activeTab="1" xr2:uid="{8AEAAAF1-D7D9-4C20-B8AF-FB019C2C5DA4}"/>
   </bookViews>
@@ -864,7 +864,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -1423,24 +1423,23 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="33" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="33" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="13" fillId="33" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="34" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="33" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="34" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1488,10 +1487,7 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <numFmt numFmtId="165" formatCode="#,##0.00\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1500,7 +1496,10 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1565,8 +1564,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{AE1F396B-21B3-47BD-9869-626466D2AECA}" name="candidatas_con_clusters__3" displayName="candidatas_con_clusters__3" ref="A1:H243" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:H243" xr:uid="{AE1F396B-21B3-47BD-9869-626466D2AECA}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{9675F67F-9EC7-4F19-9E68-71260B598FEC}" uniqueName="1" name="ticker" queryTableFieldId="1" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{843DF9CB-847B-4AA2-938B-1B7D313FE215}" uniqueName="2" name="sector" queryTableFieldId="2" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{9675F67F-9EC7-4F19-9E68-71260B598FEC}" uniqueName="1" name="ticker" queryTableFieldId="1" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{843DF9CB-847B-4AA2-938B-1B7D313FE215}" uniqueName="2" name="sector" queryTableFieldId="2" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{30B7FE35-1D76-4700-B49C-B9BD793B45BE}" uniqueName="3" name="roe" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{619F15B5-7885-459D-9816-1ADCEE438496}" uniqueName="4" name="net_profit_margin" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{C9261753-8FE3-4C82-9866-095205407047}" uniqueName="5" name="debt_to_equity" queryTableFieldId="5"/>
@@ -1582,19 +1581,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6A14E951-3E9F-40FC-8FA4-24BF9697EC37}" name="cartera_final_20empresas__3" displayName="cartera_final_20empresas__3" ref="A1:K21" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:K21" xr:uid="{6A14E951-3E9F-40FC-8FA4-24BF9697EC37}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{9AB4C27E-4F4B-4CD9-9E58-72B9EFC80A56}" uniqueName="1" name="ticker" queryTableFieldId="1" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{E1D4AD6F-2EA7-49A4-94FD-655F05CC4A49}" uniqueName="2" name="sector" queryTableFieldId="2" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{2B70A2F0-4CE4-49B7-BBE7-E64E782CA87B}" uniqueName="3" name="cluster" queryTableFieldId="3" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{9AB4C27E-4F4B-4CD9-9E58-72B9EFC80A56}" uniqueName="1" name="ticker" queryTableFieldId="1" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{E1D4AD6F-2EA7-49A4-94FD-655F05CC4A49}" uniqueName="2" name="sector" queryTableFieldId="2" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{2B70A2F0-4CE4-49B7-BBE7-E64E782CA87B}" uniqueName="3" name="cluster" queryTableFieldId="3" dataDxfId="5"/>
     <tableColumn id="4" xr3:uid="{9824D0FC-9DFF-4688-954F-F1763B1C94B5}" uniqueName="4" name="roe" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{B18F481B-38D3-4E37-BDBC-95AFD6426684}" uniqueName="5" name="net_profit_margin" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{996E3606-B94E-4215-9EB2-2F923476CED0}" uniqueName="6" name="debt_to_equity" queryTableFieldId="6"/>
     <tableColumn id="7" xr3:uid="{D46F745C-E47D-4801-A76C-E57BC85C4EAA}" uniqueName="7" name="pe_ratio" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{0E1F74AE-FE64-44A2-A19E-6550C68ED766}" uniqueName="8" name="revenue_growth" queryTableFieldId="8"/>
     <tableColumn id="9" xr3:uid="{42E1AAAC-91AE-469A-AA54-46AF7959CC65}" uniqueName="9" name="score_total" queryTableFieldId="9"/>
-    <tableColumn id="10" xr3:uid="{6B3EB127-8781-4A0A-81AB-C8533C565114}" uniqueName="10" name="peso_%" queryTableFieldId="10" dataDxfId="1">
+    <tableColumn id="10" xr3:uid="{6B3EB127-8781-4A0A-81AB-C8533C565114}" uniqueName="10" name="peso_%" queryTableFieldId="10" dataDxfId="4">
       <calculatedColumnFormula>I2/SUM($I$2:$I$21)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{9062EB8C-873A-4DF7-AA74-A76F80F3B5A4}" uniqueName="11" name="inversion_eur" queryTableFieldId="11" dataDxfId="0">
+    <tableColumn id="11" xr3:uid="{9062EB8C-873A-4DF7-AA74-A76F80F3B5A4}" uniqueName="11" name="inversion_eur" queryTableFieldId="11" dataDxfId="3">
       <calculatedColumnFormula>ROUND(J2*50000,2)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1613,7 +1612,7 @@
     <tableColumn id="5" xr3:uid="{BCC27904-87B7-4EE7-984A-59697F315AA4}" name="debt_to_equity"/>
     <tableColumn id="6" xr3:uid="{80D07911-5625-4879-B9EB-9DE358643A21}" name="pe_ratio"/>
     <tableColumn id="7" xr3:uid="{96AEB36B-4EE1-4F54-A61E-64775DB0417E}" name="revenue_growth"/>
-    <tableColumn id="8" xr3:uid="{9006945E-DC6E-4C02-A05F-E0D2739478BD}" name="cluster" dataDxfId="5">
+    <tableColumn id="8" xr3:uid="{9006945E-DC6E-4C02-A05F-E0D2739478BD}" name="cluster" dataDxfId="0">
       <calculatedColumnFormula>_xlfn.XLOOKUP(A2,candidatas_con_clusters__3[ticker],candidatas_con_clusters__3[cluster],"No encontrado")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8279,7 +8278,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CEBE3B1-E637-43B0-83C6-69E55FF1D124}">
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
@@ -8291,11 +8290,11 @@
     <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" style="3" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8323,21 +8322,21 @@
       <c r="I1" t="s">
         <v>254</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>255</v>
       </c>
       <c r="D2">
@@ -8358,23 +8357,23 @@
       <c r="I2">
         <v>0.40579999999999999</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <f t="shared" ref="J2:J21" si="0">I2/SUM($I$2:$I$21)</f>
         <v>4.2869669022491265E-2</v>
       </c>
-      <c r="K2" s="3">
+      <c r="K2" s="2">
         <f t="shared" ref="K2:K21" si="1">ROUND(J2*50000,2)</f>
         <v>2143.48</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>255</v>
       </c>
       <c r="D3">
@@ -8395,23 +8394,28 @@
       <c r="I3">
         <v>0.39340000000000003</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <f t="shared" si="0"/>
         <v>4.1559703778827173E-2</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3" s="2">
         <f t="shared" si="1"/>
         <v>2077.9899999999998</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="M3" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="N3" s="7"/>
+      <c r="O3" s="8"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>255</v>
       </c>
       <c r="D4">
@@ -8432,23 +8436,31 @@
       <c r="I4">
         <v>0.3705</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <f t="shared" si="0"/>
         <v>3.9140493772382982E-2</v>
       </c>
-      <c r="K4" s="3">
+      <c r="K4" s="2">
         <f t="shared" si="1"/>
         <v>1957.02</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="M4" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="N4" s="10"/>
+      <c r="O4" s="11">
+        <f>SUM($K$2:$K$21)</f>
+        <v>50000.000000000007</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>255</v>
       </c>
       <c r="D5">
@@ -8469,23 +8481,31 @@
       <c r="I5">
         <v>0.308</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <f t="shared" si="0"/>
         <v>3.2537846374882481E-2</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="2">
         <f t="shared" si="1"/>
         <v>1626.89</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="M5" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="N5" s="13"/>
+      <c r="O5" s="14">
+        <f>COUNT($K$2:$K$21)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>255</v>
       </c>
       <c r="D6">
@@ -8506,23 +8526,31 @@
       <c r="I6">
         <v>0.25690000000000002</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <f t="shared" si="0"/>
         <v>2.7139521862686072E-2</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="2">
         <f t="shared" si="1"/>
         <v>1356.98</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="M6" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="N6" s="10"/>
+      <c r="O6" s="15">
+        <f>ROUND(SUMPRODUCT($J$2:$J$21,$D$2:$D$21),4)</f>
+        <v>0.27489999999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>256</v>
       </c>
       <c r="D7">
@@ -8543,23 +8571,31 @@
       <c r="I7">
         <v>0.53149999999999997</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <f t="shared" si="0"/>
         <v>5.6148913468344275E-2</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K7" s="2">
         <f t="shared" si="1"/>
         <v>2807.45</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="M7" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="N7" s="13"/>
+      <c r="O7" s="14">
+        <f>ROUND(SUMPRODUCT($J$2:$J$21,$E$2:$E$21),4)</f>
+        <v>0.37340000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>117</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>256</v>
       </c>
       <c r="D8">
@@ -8580,23 +8616,31 @@
       <c r="I8">
         <v>0.48559999999999998</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <f t="shared" si="0"/>
         <v>5.1299929219619907E-2</v>
       </c>
-      <c r="K8" s="3">
+      <c r="K8" s="2">
         <f t="shared" si="1"/>
         <v>2565</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="M8" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="N8" s="4"/>
+      <c r="O8" s="5">
+        <f>ROUND(SUMPRODUCT($J$2:$J$21,$F$2:$F$21),4)</f>
+        <v>0.25640000000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>99</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>256</v>
       </c>
       <c r="D9">
@@ -8617,23 +8661,23 @@
       <c r="I9">
         <v>0.47299999999999998</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <f t="shared" si="0"/>
         <v>4.9968835504283805E-2</v>
       </c>
-      <c r="K9" s="3">
+      <c r="K9" s="2">
         <f t="shared" si="1"/>
         <v>2498.44</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>97</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>256</v>
       </c>
       <c r="D10">
@@ -8654,23 +8698,23 @@
       <c r="I10">
         <v>0.46629999999999999</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <f t="shared" si="0"/>
         <v>4.9261031703271757E-2</v>
       </c>
-      <c r="K10" s="3">
+      <c r="K10" s="2">
         <f t="shared" si="1"/>
         <v>2463.0500000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>102</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>255</v>
       </c>
       <c r="D11">
@@ -8691,23 +8735,23 @@
       <c r="I11">
         <v>0.40189999999999998</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <f t="shared" si="0"/>
         <v>4.2457663824887235E-2</v>
       </c>
-      <c r="K11" s="3">
+      <c r="K11" s="2">
         <f t="shared" si="1"/>
         <v>2122.88</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>122</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>123</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>256</v>
       </c>
       <c r="D12">
@@ -8728,23 +8772,23 @@
       <c r="I12">
         <v>0.70289999999999997</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <f t="shared" si="0"/>
         <v>7.4256013691249664E-2</v>
       </c>
-      <c r="K12" s="3">
+      <c r="K12" s="2">
         <f t="shared" si="1"/>
         <v>3712.8</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>136</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>123</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>256</v>
       </c>
       <c r="D13">
@@ -8765,23 +8809,23 @@
       <c r="I13">
         <v>0.64359999999999995</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <f t="shared" si="0"/>
         <v>6.7991421840501179E-2</v>
       </c>
-      <c r="K13" s="3">
+      <c r="K13" s="2">
         <f t="shared" si="1"/>
         <v>3399.57</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>126</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>123</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>256</v>
       </c>
       <c r="D14">
@@ -8802,23 +8846,23 @@
       <c r="I14">
         <v>0.55959999999999999</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <f t="shared" si="0"/>
         <v>5.9117463738260503E-2</v>
       </c>
-      <c r="K14" s="3">
+      <c r="K14" s="2">
         <f t="shared" si="1"/>
         <v>2955.87</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>141</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>123</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>256</v>
       </c>
       <c r="D15">
@@ -8839,23 +8883,23 @@
       <c r="I15">
         <v>0.4869</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <f t="shared" si="0"/>
         <v>5.1437264285487921E-2</v>
       </c>
-      <c r="K15" s="3">
+      <c r="K15" s="2">
         <f t="shared" si="1"/>
         <v>2571.86</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>139</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>123</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>256</v>
       </c>
       <c r="D16">
@@ -8876,23 +8920,23 @@
       <c r="I16">
         <v>0.47689999999999999</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <f t="shared" si="0"/>
         <v>5.0380840701887843E-2</v>
       </c>
-      <c r="K16" s="3">
+      <c r="K16" s="2">
         <f t="shared" si="1"/>
         <v>2519.04</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>183</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>177</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>256</v>
       </c>
       <c r="D17">
@@ -8913,23 +8957,23 @@
       <c r="I17">
         <v>0.63529999999999998</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <f t="shared" si="0"/>
         <v>6.7114590266113119E-2</v>
       </c>
-      <c r="K17" s="3">
+      <c r="K17" s="2">
         <f t="shared" si="1"/>
         <v>3355.73</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>200</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>177</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>256</v>
       </c>
       <c r="D18">
@@ -8950,23 +8994,23 @@
       <c r="I18">
         <v>0.48509999999999998</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <f t="shared" si="0"/>
         <v>5.1247108040439901E-2</v>
       </c>
-      <c r="K18" s="3">
+      <c r="K18" s="2">
         <f t="shared" si="1"/>
         <v>2562.36</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="A19" t="s">
         <v>202</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>177</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" t="s">
         <v>256</v>
       </c>
       <c r="D19">
@@ -8987,23 +9031,23 @@
       <c r="I19">
         <v>0.47360000000000002</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <f t="shared" si="0"/>
         <v>5.0032220919299819E-2</v>
       </c>
-      <c r="K19" s="3">
+      <c r="K19" s="2">
         <f t="shared" si="1"/>
         <v>2501.61</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>176</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>177</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>255</v>
       </c>
       <c r="D20">
@@ -9024,23 +9068,23 @@
       <c r="I20">
         <v>0.46550000000000002</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <f t="shared" si="0"/>
         <v>4.9176517816583755E-2</v>
       </c>
-      <c r="K20" s="3">
+      <c r="K20" s="2">
         <f t="shared" si="1"/>
         <v>2458.83</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="A21" t="s">
         <v>181</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>177</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" t="s">
         <v>256</v>
       </c>
       <c r="D21">
@@ -9061,70 +9105,13 @@
       <c r="I21">
         <v>0.44359999999999999</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <f t="shared" si="0"/>
         <v>4.6862950168499569E-2</v>
       </c>
-      <c r="K21" s="3">
+      <c r="K21" s="2">
         <f t="shared" si="1"/>
         <v>2343.15</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="9"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>260</v>
-      </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="12">
-        <f>SUM($K$2:$K$21)</f>
-        <v>50000.000000000007</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
-        <v>259</v>
-      </c>
-      <c r="B26" s="14"/>
-      <c r="C26" s="15">
-        <f>COUNT($K$2:$K$21)</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="10" t="s">
-        <v>261</v>
-      </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="16">
-        <f>ROUND(SUMPRODUCT($J$2:$J$21,$D$2:$D$21),4)</f>
-        <v>0.27489999999999998</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
-        <v>262</v>
-      </c>
-      <c r="B28" s="14"/>
-      <c r="C28" s="15">
-        <f>ROUND(SUMPRODUCT($J$2:$J$21,$E$2:$E$21),4)</f>
-        <v>0.37340000000000001</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
-        <v>263</v>
-      </c>
-      <c r="B29" s="5"/>
-      <c r="C29" s="6">
-        <f>ROUND(SUMPRODUCT($J$2:$J$21,$F$2:$F$21),4)</f>
-        <v>0.25640000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>